<commit_message>
v13.73: docs(cupia): 견적서 수식 셀 MS Office 빈 칸 문제 수정 — 수식 캐시값 주입(빈 <v></v> → 계산값, _1 13셀·_2 14셀) + fullCalcOnLoad 설정(양식 포함), data_only 검증 합계 220,000,000원 확인
</commit_message>
<xml_diff>
--- a/cupia-ai-research/docs/08_계약관리/[CUPIA] EWACS_복합_AI_Agent_구축_견적서_20260731_1.xlsx
+++ b/cupia-ai-research/docs/08_계약관리/[CUPIA] EWACS_복합_AI_Agent_구축_견적서_20260731_1.xlsx
@@ -12,7 +12,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'견적서(인력)'!$A$1:$L$34</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
 </workbook>
 </file>
 
@@ -3725,7 +3725,7 @@
       </c>
       <c r="I17" s="107">
         <f>F17*G17*H17</f>
-        <v/>
+        <v>74543819</v>
       </c>
       <c r="J17" s="108" t="n">
         <v>0</v>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="I18" s="107">
         <f>F18*G18*H18</f>
-        <v/>
+        <v>46524744</v>
       </c>
       <c r="J18" s="108" t="n">
         <v>0</v>
@@ -3795,7 +3795,7 @@
       </c>
       <c r="I19" s="107">
         <f>F19*G19*H19</f>
-        <v/>
+        <v>27606640</v>
       </c>
       <c r="J19" s="108" t="n">
         <v>0</v>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="I20" s="107">
         <f>F20*G20*H20</f>
-        <v/>
+        <v>33126213</v>
       </c>
       <c r="J20" s="108" t="n">
         <v>0</v>
@@ -3865,7 +3865,7 @@
       </c>
       <c r="I21" s="107">
         <f>F21*G21*H21</f>
-        <v/>
+        <v>11680392</v>
       </c>
       <c r="J21" s="108" t="n">
         <v>0</v>
@@ -3902,7 +3902,7 @@
       </c>
       <c r="I22" s="120">
         <f>SUM(I17:I21)</f>
-        <v/>
+        <v>193481808</v>
       </c>
       <c r="J22" s="121" t="n">
         <v>0</v>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="I23" s="127">
         <f>ROUND(I22*6%,0)</f>
-        <v/>
+        <v>11608908</v>
       </c>
       <c r="J23" s="127" t="n"/>
       <c r="K23" s="128" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="I25" s="120">
         <f>SUM(I23:I24)</f>
-        <v/>
+        <v>26518192</v>
       </c>
       <c r="J25" s="121" t="n">
         <v>0</v>
@@ -4049,11 +4049,11 @@
       </c>
       <c r="I26" s="134">
         <f>I22+I25</f>
-        <v/>
+        <v>220000000</v>
       </c>
       <c r="J26" s="134">
         <f>J22+J25</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K26" s="135" t="n"/>
     </row>
@@ -4071,11 +4071,11 @@
       <c r="H27" s="93" t="n"/>
       <c r="I27" s="138">
         <f>I26</f>
-        <v/>
+        <v>220000000</v>
       </c>
       <c r="J27" s="139">
         <f>I26</f>
-        <v/>
+        <v>220000000</v>
       </c>
       <c r="K27" s="140" t="inlineStr">
         <is>
@@ -4095,7 +4095,7 @@
       <c r="J28" s="143" t="n"/>
       <c r="K28" s="144">
         <f>100%-(J27/I27)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="29" ht="62" customHeight="1" s="72">

</xml_diff>